<commit_message>
SUMMARY OD STUDIO BUSINESS REPORT
</commit_message>
<xml_diff>
--- a/admin_v2/ROYALTY_SERVICE_REPORT.xlsx
+++ b/admin_v2/ROYALTY_SERVICE_REPORT.xlsx
@@ -20,13 +20,13 @@
     <t>ROYALTY SERVICE REPORT</t>
   </si>
   <si>
-    <t>Franchisee: Amto.Robert (Arthur Murray Thousand Oaks)</t>
-  </si>
-  <si>
-    <t>(09/14/2025 - 09/20/2025)</t>
-  </si>
-  <si>
-    <t>Week # 38</t>
+    <t xml:space="preserve"> (Bidyanandapur, Arthur Murray Woodland Hills, sdgh, location, gggggggggg)</t>
+  </si>
+  <si>
+    <t>(12/31/1969 - 01/06/1970)</t>
+  </si>
+  <si>
+    <t>Week # 28</t>
   </si>
   <si>
     <t>Staff code</t>

</xml_diff>